<commit_message>
calibracion: politica propuesta con restriccion de capital neutral
</commit_message>
<xml_diff>
--- a/resultados/caso_negocio.xlsx
+++ b/resultados/caso_negocio.xlsx
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="B6" s="11" t="n">
-        <v>209435.0483493663</v>
+        <v>186330.8138987838</v>
       </c>
     </row>
     <row r="7">
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>2.584319719232242</v>
+        <v>1.417976287872458</v>
       </c>
     </row>
     <row r="8">
@@ -848,7 +848,7 @@
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>2.238137739177289</v>
+        <v>1.147670941575063</v>
       </c>
     </row>
     <row r="9">
@@ -880,7 +880,7 @@
         </is>
       </c>
       <c r="B11" s="11" t="n">
-        <v>8096.507586195687</v>
+        <v>118.6677464388777</v>
       </c>
     </row>
     <row r="12">
@@ -1059,7 +1059,7 @@
         </is>
       </c>
       <c r="B31" s="11" t="n">
-        <v>1619832.79</v>
+        <v>1388166.29</v>
       </c>
     </row>
     <row r="32">
@@ -1069,7 +1069,7 @@
         </is>
       </c>
       <c r="B32" s="11" t="n">
-        <v>564389.13</v>
+        <v>274778.85</v>
       </c>
     </row>
     <row r="33">
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="B33" s="11" t="n">
-        <v>800082.11</v>
+        <v>800599.7</v>
       </c>
     </row>
     <row r="34">
@@ -1089,7 +1089,7 @@
         </is>
       </c>
       <c r="B34" s="11" t="n">
-        <v>-21760.39</v>
+        <v>-298.06</v>
       </c>
     </row>
     <row r="35">
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>114513</v>
+        <v>105007</v>
       </c>
       <c r="C4" s="4">
         <f>Supuestos!$B$5</f>
@@ -1192,7 +1192,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>39899.11</v>
+        <v>20785.48</v>
       </c>
       <c r="C5" s="4">
         <f>Supuestos!$B$5</f>
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>56561.27</v>
+        <v>60560.88</v>
       </c>
       <c r="C6" s="4">
         <f>Supuestos!$B$5</f>
@@ -1236,7 +1236,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-1538.34</v>
+        <v>-22.55</v>
       </c>
       <c r="C7" s="4">
         <f>Supuestos!$B$5</f>

</xml_diff>

<commit_message>
funcionalidad: informes, tablero, pruebas y sitio de portafolio
</commit_message>
<xml_diff>
--- a/resultados/caso_negocio.xlsx
+++ b/resultados/caso_negocio.xlsx
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="B6" s="11" t="n">
-        <v>186330.8138987838</v>
+        <v>182435.3758513053</v>
       </c>
     </row>
     <row r="7">
@@ -838,7 +838,7 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>1.417976287872458</v>
+        <v>1.299653704218329</v>
       </c>
     </row>
     <row r="8">
@@ -848,7 +848,7 @@
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>1.147670941575063</v>
+        <v>1.824097437638433</v>
       </c>
     </row>
     <row r="9">
@@ -880,7 +880,7 @@
         </is>
       </c>
       <c r="B11" s="11" t="n">
-        <v>118.6677464388777</v>
+        <v>-157.3423205131839</v>
       </c>
     </row>
     <row r="12">
@@ -1059,7 +1059,7 @@
         </is>
       </c>
       <c r="B31" s="11" t="n">
-        <v>1388166.29</v>
+        <v>1703566.67</v>
       </c>
     </row>
     <row r="32">
@@ -1069,7 +1069,7 @@
         </is>
       </c>
       <c r="B32" s="11" t="n">
-        <v>274778.85</v>
+        <v>276037.01</v>
       </c>
     </row>
     <row r="33">
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="B33" s="11" t="n">
-        <v>800599.7</v>
+        <v>999685.84</v>
       </c>
     </row>
     <row r="34">
@@ -1089,7 +1089,7 @@
         </is>
       </c>
       <c r="B34" s="11" t="n">
-        <v>-298.06</v>
+        <v>488.29</v>
       </c>
     </row>
     <row r="35">
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>105007</v>
+        <v>104300</v>
       </c>
       <c r="C4" s="4">
         <f>Supuestos!$B$5</f>
@@ -1192,7 +1192,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>20785.48</v>
+        <v>16900.23</v>
       </c>
       <c r="C5" s="4">
         <f>Supuestos!$B$5</f>
@@ -1214,7 +1214,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>60560.88</v>
+        <v>61205.26</v>
       </c>
       <c r="C6" s="4">
         <f>Supuestos!$B$5</f>
@@ -1236,7 +1236,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-22.55</v>
+        <v>29.9</v>
       </c>
       <c r="C7" s="4">
         <f>Supuestos!$B$5</f>

</xml_diff>